<commit_message>
Update para coluna de usuários inativos no sistema para NDE e IMP 008
</commit_message>
<xml_diff>
--- a/qstione/nde/nde.xlsx
+++ b/qstione/nde/nde.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonardo.paiva\aluno-sync\qstione\nde\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB358CC7-A474-4A7F-83BC-48A80C3E070C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA89F12E-88C7-40B0-B175-A52196E05145}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="18855" windowHeight="12690" xr2:uid="{1D63BFA0-2A1E-47B9-9F61-C07C12A21ABA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1D63BFA0-2A1E-47B9-9F61-C07C12A21ABA}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="203">
   <si>
     <t>Coordenador</t>
   </si>
@@ -300,9 +300,6 @@
     <t>DANIELE RIBEIRO DO VAL DE OLIVEIRA LIMA SANTA BARBARA</t>
   </si>
   <si>
-    <t>MARCOS AURELIO RAMALHO GANDRA</t>
-  </si>
-  <si>
     <t>MONICA SANTOS BARISON</t>
   </si>
   <si>
@@ -591,9 +588,6 @@
     <t>daniele.barbara@foa.org.br</t>
   </si>
   <si>
-    <t>marcos.gandra@foa.org.br</t>
-  </si>
-  <si>
     <t>monica.barison@foa.org.br</t>
   </si>
   <si>
@@ -637,13 +631,31 @@
   </si>
   <si>
     <t>venicio.siqueira@foa.org.br</t>
+  </si>
+  <si>
+    <t>eduardo.miranda@foa.org.br</t>
+  </si>
+  <si>
+    <t>julio.nobre@foa.org.br</t>
+  </si>
+  <si>
+    <t>aline.reboucas@foa.org.br</t>
+  </si>
+  <si>
+    <t>bruna.casiraghi@foa.org.br</t>
+  </si>
+  <si>
+    <t>sonia.garcia@foa.org.br</t>
+  </si>
+  <si>
+    <t>145</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -672,6 +684,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -690,10 +710,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
@@ -710,8 +731,16 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1038,36 +1067,36 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -1078,10 +1107,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>2</v>
@@ -1095,10 +1124,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>2</v>
@@ -1112,10 +1141,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>2</v>
@@ -1129,16 +1158,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>12</v>
@@ -1149,10 +1178,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>11</v>
@@ -1166,10 +1195,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>11</v>
@@ -1183,10 +1212,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>11</v>
@@ -1200,16 +1229,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>3</v>
@@ -1220,10 +1249,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>2</v>
@@ -1237,10 +1266,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>2</v>
@@ -1254,10 +1283,10 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>2</v>
@@ -1271,30 +1300,30 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>20</v>
@@ -1303,15 +1332,15 @@
         <v>22</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>20</v>
@@ -1320,15 +1349,15 @@
         <v>23</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>20</v>
@@ -1337,35 +1366,35 @@
         <v>24</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>26</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>25</v>
@@ -1374,15 +1403,15 @@
         <v>27</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>25</v>
@@ -1391,15 +1420,15 @@
         <v>28</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>25</v>
@@ -1408,15 +1437,15 @@
         <v>29</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>25</v>
@@ -1425,15 +1454,15 @@
         <v>30</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>25</v>
@@ -1442,35 +1471,35 @@
         <v>31</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>33</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>32</v>
@@ -1479,15 +1508,15 @@
         <v>34</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>32</v>
@@ -1496,15 +1525,15 @@
         <v>35</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>32</v>
@@ -1513,15 +1542,15 @@
         <v>36</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>32</v>
@@ -1530,21 +1559,21 @@
         <v>37</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>38</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>39</v>
@@ -1555,10 +1584,10 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>38</v>
@@ -1572,10 +1601,10 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>38</v>
@@ -1589,10 +1618,10 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>38</v>
@@ -1606,10 +1635,10 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>38</v>
@@ -1623,30 +1652,30 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>55</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>50</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>55</v>
@@ -1655,15 +1684,15 @@
         <v>51</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>55</v>
@@ -1672,15 +1701,15 @@
         <v>52</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>55</v>
@@ -1689,15 +1718,15 @@
         <v>53</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>55</v>
@@ -1706,35 +1735,35 @@
         <v>54</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>56</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>50</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>56</v>
@@ -1743,15 +1772,15 @@
         <v>51</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>56</v>
@@ -1760,15 +1789,15 @@
         <v>52</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>56</v>
@@ -1777,15 +1806,15 @@
         <v>53</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>56</v>
@@ -1794,35 +1823,35 @@
         <v>54</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>49</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>50</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>49</v>
@@ -1831,15 +1860,15 @@
         <v>51</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>49</v>
@@ -1848,15 +1877,15 @@
         <v>52</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>49</v>
@@ -1865,15 +1894,15 @@
         <v>53</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>49</v>
@@ -1882,35 +1911,35 @@
         <v>54</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>57</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>50</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>57</v>
@@ -1919,15 +1948,15 @@
         <v>51</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>57</v>
@@ -1936,15 +1965,15 @@
         <v>52</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>57</v>
@@ -1953,15 +1982,15 @@
         <v>53</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>57</v>
@@ -1970,35 +1999,35 @@
         <v>54</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>57</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>50</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>57</v>
@@ -2007,15 +2036,15 @@
         <v>51</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>57</v>
@@ -2024,15 +2053,15 @@
         <v>52</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>57</v>
@@ -2041,15 +2070,15 @@
         <v>53</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>57</v>
@@ -2058,35 +2087,35 @@
         <v>54</v>
       </c>
       <c r="F58" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>58</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F59" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>58</v>
@@ -2095,15 +2124,15 @@
         <v>60</v>
       </c>
       <c r="F60" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>58</v>
@@ -2112,15 +2141,15 @@
         <v>61</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>58</v>
@@ -2129,15 +2158,15 @@
         <v>62</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>58</v>
@@ -2146,35 +2175,35 @@
         <v>63</v>
       </c>
       <c r="F63" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>64</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>65</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>64</v>
@@ -2183,15 +2212,15 @@
         <v>66</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>64</v>
@@ -2200,15 +2229,15 @@
         <v>67</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>64</v>
@@ -2217,35 +2246,35 @@
         <v>68</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>69</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>70</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>69</v>
@@ -2254,15 +2283,15 @@
         <v>71</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>69</v>
@@ -2271,15 +2300,15 @@
         <v>72</v>
       </c>
       <c r="F70" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>69</v>
@@ -2288,15 +2317,15 @@
         <v>73</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>69</v>
@@ -2305,15 +2334,15 @@
         <v>74</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B73" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>69</v>
@@ -2322,15 +2351,15 @@
         <v>75</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B74" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>69</v>
@@ -2339,21 +2368,33 @@
         <v>76</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>202</v>
+      </c>
       <c r="B75" s="1" t="s">
         <v>77</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="D75" s="1" t="s">
+        <v>197</v>
+      </c>
       <c r="E75" s="1" t="s">
         <v>79</v>
       </c>
+      <c r="F75" s="7" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>202</v>
+      </c>
       <c r="B76" s="1" t="s">
         <v>77</v>
       </c>
@@ -2363,8 +2404,14 @@
       <c r="E76" s="1" t="s">
         <v>80</v>
       </c>
+      <c r="F76" s="7" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>202</v>
+      </c>
       <c r="B77" s="1" t="s">
         <v>77</v>
       </c>
@@ -2374,8 +2421,14 @@
       <c r="E77" s="1" t="s">
         <v>78</v>
       </c>
+      <c r="F77" s="1" t="s">
+        <v>197</v>
+      </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>202</v>
+      </c>
       <c r="B78" s="1" t="s">
         <v>77</v>
       </c>
@@ -2385,8 +2438,14 @@
       <c r="E78" s="1" t="s">
         <v>81</v>
       </c>
+      <c r="F78" s="6" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>202</v>
+      </c>
       <c r="B79" s="1" t="s">
         <v>77</v>
       </c>
@@ -2396,33 +2455,36 @@
       <c r="E79" s="1" t="s">
         <v>82</v>
       </c>
+      <c r="F79" s="7" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>58</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B81" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>58</v>
@@ -2431,15 +2493,15 @@
         <v>60</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B82" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>58</v>
@@ -2448,15 +2510,15 @@
         <v>61</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B83" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>58</v>
@@ -2465,15 +2527,15 @@
         <v>62</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B84" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>58</v>
@@ -2482,35 +2544,35 @@
         <v>63</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B85" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>83</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E85" s="1" t="s">
         <v>84</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>83</v>
@@ -2519,153 +2581,153 @@
         <v>85</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B87" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>83</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F87" s="3" t="s">
-        <v>183</v>
+        <v>81</v>
+      </c>
+      <c r="F87" s="6" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="B88" s="1" t="s">
         <v>132</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="C88" s="1" t="s">
         <v>83</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B89" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B89" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="C89" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E89" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="D89" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="E89" s="1" t="s">
-        <v>89</v>
-      </c>
       <c r="F89" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B90" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B90" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="C90" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B91" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="C91" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F91" s="3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B92" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="C92" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F92" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B93" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="B93" s="1" t="s">
-        <v>135</v>
-      </c>
       <c r="C93" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B96" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -2675,6 +2737,14 @@
     </sortState>
   </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="F87" r:id="rId1" xr:uid="{E6DDA6F2-0DC8-469A-BCA7-5994C73ABAAF}"/>
+    <hyperlink ref="F78" r:id="rId2" xr:uid="{8B7277B2-E321-40C0-977A-008E52798ED5}"/>
+    <hyperlink ref="F75" r:id="rId3" display="mailto:ALINE.REBOUCAS@FOA.ORG.BR" xr:uid="{0AFF214C-4262-4469-863F-BD5CCCF52561}"/>
+    <hyperlink ref="F76" r:id="rId4" display="mailto:BRUNA.CASIRAGHI@FOA.ORG.BR" xr:uid="{D136B2A8-0875-4A47-9E32-4107867B0C39}"/>
+    <hyperlink ref="F79" r:id="rId5" xr:uid="{B271E94E-7C03-4040-8115-1B0096050A10}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>